<commit_message>
feat: new version 1.1.0 with remastered UX/UI
</commit_message>
<xml_diff>
--- a/docs/2026-suivi-missions-argent-de-poche.xlsx
+++ b/docs/2026-suivi-missions-argent-de-poche.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="missions_hiver" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="missions_printemps" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="missions_ete" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="missions_automne" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bilan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="missions_hiver" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="missions_printemps" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="missions_ete" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="missions_automne" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="bilan" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -757,7 +757,7 @@
     </row>
     <row r="2" ht="22.5" customHeight="1" s="16">
       <c r="A2" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="13" t="n">
         <v>46115</v>
@@ -1339,7 +1339,7 @@
     </row>
     <row r="8" ht="22.5" customHeight="1" s="16">
       <c r="A8" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
@@ -1471,7 +1471,7 @@
     </row>
     <row r="10" ht="22.5" customHeight="1" s="16">
       <c r="A10" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
@@ -1603,7 +1603,7 @@
     </row>
     <row r="12" ht="22.5" customHeight="1" s="16">
       <c r="A12" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
@@ -1669,7 +1669,7 @@
     </row>
     <row r="13" ht="22.5" customHeight="1" s="16">
       <c r="A13" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
@@ -1735,7 +1735,7 @@
     </row>
     <row r="14" ht="22.5" customHeight="1" s="16">
       <c r="A14" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
@@ -1801,7 +1801,7 @@
     </row>
     <row r="15" ht="22.5" customHeight="1" s="16">
       <c r="A15" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
@@ -1867,7 +1867,7 @@
     </row>
     <row r="16" ht="22.5" customHeight="1" s="16">
       <c r="A16" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
@@ -1933,7 +1933,7 @@
     </row>
     <row r="17" ht="22.5" customHeight="1" s="16">
       <c r="A17" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
@@ -1999,7 +1999,7 @@
     </row>
     <row r="18" ht="22.5" customHeight="1" s="16">
       <c r="A18" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="19" ht="22.5" customHeight="1" s="16">
       <c r="A19" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
@@ -2131,7 +2131,7 @@
     </row>
     <row r="20" ht="22.5" customHeight="1" s="16">
       <c r="A20" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
@@ -2197,7 +2197,7 @@
     </row>
     <row r="21" ht="15.75" customHeight="1" s="16">
       <c r="A21" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
     </row>
     <row r="22" ht="15.75" customHeight="1" s="16">
       <c r="A22" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
@@ -2329,7 +2329,7 @@
     </row>
     <row r="23" ht="15.75" customHeight="1" s="16">
       <c r="A23" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
@@ -2395,7 +2395,7 @@
     </row>
     <row r="24" ht="15.75" customHeight="1" s="16">
       <c r="A24" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
@@ -2461,7 +2461,7 @@
     </row>
     <row r="25" ht="15.75" customHeight="1" s="16">
       <c r="A25" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
@@ -2527,7 +2527,7 @@
     </row>
     <row r="26" ht="15.75" customHeight="1" s="16">
       <c r="A26" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
@@ -2593,7 +2593,7 @@
     </row>
     <row r="27" ht="15.75" customHeight="1" s="16">
       <c r="A27" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
@@ -2659,7 +2659,7 @@
     </row>
     <row r="28" ht="15.75" customHeight="1" s="16">
       <c r="A28" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
@@ -2725,7 +2725,7 @@
     </row>
     <row r="29" ht="15.75" customHeight="1" s="16">
       <c r="A29" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
@@ -2791,7 +2791,7 @@
     </row>
     <row r="30" ht="15.75" customHeight="1" s="16">
       <c r="A30" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
@@ -2857,7 +2857,7 @@
     </row>
     <row r="31" ht="15.75" customHeight="1" s="16">
       <c r="A31" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     </row>
     <row r="32" ht="15.75" customHeight="1" s="16">
       <c r="A32" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
@@ -2989,7 +2989,7 @@
     </row>
     <row r="33" ht="15.75" customHeight="1" s="16">
       <c r="A33" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
@@ -3055,7 +3055,7 @@
     </row>
     <row r="34" ht="15.75" customHeight="1" s="16">
       <c r="A34" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
@@ -3121,7 +3121,7 @@
     </row>
     <row r="35" ht="15.75" customHeight="1" s="16">
       <c r="A35" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
@@ -3187,7 +3187,7 @@
     </row>
     <row r="36" ht="15.75" customHeight="1" s="16">
       <c r="A36" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
@@ -3253,7 +3253,7 @@
     </row>
     <row r="37" ht="15.75" customHeight="1" s="16">
       <c r="A37" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
@@ -3319,7 +3319,7 @@
     </row>
     <row r="38" ht="15.75" customHeight="1" s="16">
       <c r="A38" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
@@ -3385,7 +3385,7 @@
     </row>
     <row r="39" ht="15.75" customHeight="1" s="16">
       <c r="A39" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
@@ -3451,7 +3451,7 @@
     </row>
     <row r="40" ht="15.75" customHeight="1" s="16">
       <c r="A40" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
@@ -3517,7 +3517,7 @@
     </row>
     <row r="41" ht="15.75" customHeight="1" s="16">
       <c r="A41" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
@@ -3583,7 +3583,7 @@
     </row>
     <row r="42" ht="15.75" customHeight="1" s="16">
       <c r="A42" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
@@ -3649,7 +3649,7 @@
     </row>
     <row r="43" ht="15.75" customHeight="1" s="16">
       <c r="A43" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B43" s="11" t="inlineStr">
         <is>
@@ -3715,7 +3715,7 @@
     </row>
     <row r="44" ht="15.75" customHeight="1" s="16">
       <c r="A44" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
@@ -3781,7 +3781,7 @@
     </row>
     <row r="45" ht="15.75" customHeight="1" s="16">
       <c r="A45" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B45" s="11" t="inlineStr">
         <is>
@@ -3847,7 +3847,7 @@
     </row>
     <row r="46" ht="15.75" customHeight="1" s="16">
       <c r="A46" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B46" s="11" t="inlineStr">
         <is>
@@ -3913,7 +3913,7 @@
     </row>
     <row r="47" ht="15.75" customHeight="1" s="16">
       <c r="A47" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B47" s="11" t="inlineStr">
         <is>
@@ -3979,7 +3979,7 @@
     </row>
     <row r="48" ht="15.75" customHeight="1" s="16">
       <c r="A48" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
@@ -4045,7 +4045,7 @@
     </row>
     <row r="49" ht="15.75" customHeight="1" s="16">
       <c r="A49" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B49" s="11" t="inlineStr">
         <is>
@@ -4111,7 +4111,7 @@
     </row>
     <row r="50" ht="15.75" customHeight="1" s="16">
       <c r="A50" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
@@ -4177,7 +4177,7 @@
     </row>
     <row r="51" ht="15.75" customHeight="1" s="16">
       <c r="A51" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B51" s="11" t="inlineStr">
         <is>
@@ -4243,7 +4243,7 @@
     </row>
     <row r="52" ht="15.75" customHeight="1" s="16">
       <c r="A52" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
@@ -4309,7 +4309,7 @@
     </row>
     <row r="53" ht="15.75" customHeight="1" s="16">
       <c r="A53" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B53" s="11" t="inlineStr">
         <is>
@@ -4375,7 +4375,7 @@
     </row>
     <row r="54" ht="15.75" customHeight="1" s="16">
       <c r="A54" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
@@ -4441,7 +4441,7 @@
     </row>
     <row r="55" ht="15.75" customHeight="1" s="16">
       <c r="A55" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
@@ -4507,7 +4507,7 @@
     </row>
     <row r="56" ht="15.75" customHeight="1" s="16">
       <c r="A56" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
     </row>
     <row r="57" ht="15.75" customHeight="1" s="16">
       <c r="A57" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
@@ -4639,7 +4639,7 @@
     </row>
     <row r="58" ht="15.75" customHeight="1" s="16">
       <c r="A58" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
@@ -4705,7 +4705,7 @@
     </row>
     <row r="59" ht="15.75" customHeight="1" s="16">
       <c r="A59" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B59" s="11" t="inlineStr">
         <is>
@@ -4771,7 +4771,7 @@
     </row>
     <row r="60" ht="15.75" customHeight="1" s="16">
       <c r="A60" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B60" s="11" t="inlineStr">
         <is>
@@ -4837,7 +4837,7 @@
     </row>
     <row r="61" ht="15.75" customHeight="1" s="16">
       <c r="A61" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B61" s="11" t="inlineStr">
         <is>
@@ -4903,7 +4903,7 @@
     </row>
     <row r="62" ht="15.75" customHeight="1" s="16">
       <c r="A62" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
@@ -4969,7 +4969,7 @@
     </row>
     <row r="63" ht="15.75" customHeight="1" s="16">
       <c r="A63" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B63" s="11" t="inlineStr">
         <is>
@@ -5035,7 +5035,7 @@
     </row>
     <row r="64" ht="15.75" customHeight="1" s="16">
       <c r="A64" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B64" s="11" t="inlineStr">
         <is>
@@ -5101,7 +5101,7 @@
     </row>
     <row r="65" ht="15.75" customHeight="1" s="16">
       <c r="A65" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B65" s="11" t="inlineStr">
         <is>
@@ -5167,7 +5167,7 @@
     </row>
     <row r="66" ht="15.75" customHeight="1" s="16">
       <c r="A66" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B66" s="11" t="inlineStr">
         <is>
@@ -5233,7 +5233,7 @@
     </row>
     <row r="67" ht="15.75" customHeight="1" s="16">
       <c r="A67" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B67" s="11" t="inlineStr">
         <is>
@@ -5299,7 +5299,7 @@
     </row>
     <row r="68" ht="15.75" customHeight="1" s="16">
       <c r="A68" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B68" s="11" t="inlineStr">
         <is>
@@ -5365,7 +5365,7 @@
     </row>
     <row r="69" ht="15.75" customHeight="1" s="16">
       <c r="A69" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B69" s="11" t="inlineStr">
         <is>
@@ -5431,7 +5431,7 @@
     </row>
     <row r="70" ht="15.75" customHeight="1" s="16">
       <c r="A70" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B70" s="11" t="inlineStr">
         <is>
@@ -5497,7 +5497,7 @@
     </row>
     <row r="71" ht="15.75" customHeight="1" s="16">
       <c r="A71" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B71" s="11" t="inlineStr">
         <is>
@@ -5563,7 +5563,7 @@
     </row>
     <row r="72" ht="15.75" customHeight="1" s="16">
       <c r="A72" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
@@ -5629,7 +5629,7 @@
     </row>
     <row r="73" ht="15.75" customHeight="1" s="16">
       <c r="A73" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B73" s="11" t="inlineStr">
         <is>
@@ -5695,7 +5695,7 @@
     </row>
     <row r="74" ht="15.75" customHeight="1" s="16">
       <c r="A74" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B74" s="11" t="inlineStr">
         <is>
@@ -5761,7 +5761,7 @@
     </row>
     <row r="75" ht="15.75" customHeight="1" s="16">
       <c r="A75" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B75" s="11" t="inlineStr">
         <is>
@@ -5827,7 +5827,7 @@
     </row>
     <row r="76" ht="15.75" customHeight="1" s="16">
       <c r="A76" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B76" s="11" t="inlineStr">
         <is>
@@ -5893,7 +5893,7 @@
     </row>
     <row r="77" ht="15.75" customHeight="1" s="16">
       <c r="A77" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B77" s="11" t="inlineStr">
         <is>
@@ -5959,7 +5959,7 @@
     </row>
     <row r="78" ht="15.75" customHeight="1" s="16">
       <c r="A78" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B78" s="11" t="inlineStr">
         <is>
@@ -6025,7 +6025,7 @@
     </row>
     <row r="79" ht="15.75" customHeight="1" s="16">
       <c r="A79" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B79" s="11" t="inlineStr">
         <is>
@@ -6091,7 +6091,7 @@
     </row>
     <row r="80" ht="15.75" customHeight="1" s="16">
       <c r="A80" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B80" s="11" t="inlineStr">
         <is>
@@ -6157,7 +6157,7 @@
     </row>
     <row r="81" ht="15.75" customHeight="1" s="16">
       <c r="A81" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B81" s="11" t="inlineStr">
         <is>
@@ -6223,7 +6223,7 @@
     </row>
     <row r="82" ht="15.75" customHeight="1" s="16">
       <c r="A82" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B82" s="11" t="inlineStr">
         <is>
@@ -6289,7 +6289,7 @@
     </row>
     <row r="83" ht="15.75" customHeight="1" s="16">
       <c r="A83" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
@@ -6355,7 +6355,7 @@
     </row>
     <row r="84" ht="15.75" customHeight="1" s="16">
       <c r="A84" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
@@ -6421,7 +6421,7 @@
     </row>
     <row r="85" ht="15.75" customHeight="1" s="16">
       <c r="A85" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
@@ -6487,7 +6487,7 @@
     </row>
     <row r="86" ht="15.75" customHeight="1" s="16">
       <c r="A86" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B86" s="11" t="inlineStr">
         <is>
@@ -6553,7 +6553,7 @@
     </row>
     <row r="87" ht="15.75" customHeight="1" s="16">
       <c r="A87" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B87" s="11" t="inlineStr">
         <is>
@@ -6619,7 +6619,7 @@
     </row>
     <row r="88" ht="15.75" customHeight="1" s="16">
       <c r="A88" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B88" s="11" t="inlineStr">
         <is>

</xml_diff>